<commit_message>
feat: robots.txt/sitemap 점검 항목 추가 (메인 홈), 점검결과 403 반영
- robots.txt 실측: www·m.hanwhadirect.com/robots.txt 모두 HTTP 403(봇 차단)
- 홈(메인 m.hanwhadirect.com) To-Do에 robots.txt·sitemap 설치/점검 추가(우선순위 상)
  · Yeti·Googlebot 명시 허용 + Sitemap 등록 권장본 제공
- 기존 홈 JSON-LD 항목은 robots로 대체(순수 파일/HTML 위주)
- Excel/PPT 태깅가이드도 동일 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhxZYksEXdBzqoiFpg6L1A
</commit_message>
<xml_diff>
--- a/handoff/한화손보_장기CM_태깅가이드.xlsx
+++ b/handoff/한화손보_장기CM_태깅가이드.xlsx
@@ -1321,22 +1321,77 @@
           <t>https://m.hanwhadirect.com/</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>robots.txt · sitemap.xml 설치/점검 (사이트 전체)</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t># https://www.hanwhadirect.com/robots.txt → 현재 403 (설치·크롤러 허용 여부 확인 필요)</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t># robots.txt (사이트 루트)
+User-agent: Yeti
+Allow: /
+User-agent: Googlebot
+Allow: /
+User-agent: *
+Allow: /
+Sitemap: https://www.hanwhadirect.com/sitemap.xml</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr"/>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>H1·alt·OG 원본은 실제 DOM 확인 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>다이렉트 홈(메인)</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>한화손보다이렉트</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>메인</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>https://m.hanwhadirect.com/</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>중</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>OG 태그 세트 추가/점검</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>&lt;!-- og:* 태그 없음/부분 --&gt;</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>&lt;meta property="og:title" content="한화손보다이렉트 — 필요한 보험을 한 곳에서"&gt;
 &lt;meta property="og:description" content="장기보험을 개인정보 없이 3분 만에 비교하고 보험료를 확인해요."&gt;
@@ -1344,101 +1399,53 @@
 &lt;meta property="og:url" content="https://m.hanwhadirect.com/"&gt;</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr"/>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr"/>
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>H1·alt·OG 원본은 실제 DOM 확인 후</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>다이렉트 홈(메인)</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>한화손보다이렉트</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>메인</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>https://m.hanwhadirect.com/</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>중</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>모바일(m.)·PC(www) 메타 일치 + canonical</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>&lt;!-- m./www 메타 상이·canonical 누락 가능 --&gt;</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>&lt;link rel="canonical" href="https://www.hanwhadirect.com/"&gt;
 &lt;link rel="alternate" media="only screen and (max-width: 640px)" href="https://m.hanwhadirect.com/"&gt;</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr"/>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>H1·alt·OG 원본은 실제 DOM 확인 후</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>다이렉트 홈(메인)</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>한화손보다이렉트</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>메인</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>https://m.hanwhadirect.com/</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>사이트명·브랜드 구조화(WebSite/Organization)</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>&lt;!-- WebSite/Organization 구조화 없음 --&gt;</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>&lt;script type="application/ld+json"&gt;{"@context":"https://schema.org","@type":"WebSite","name":"한화손해보험 다이렉트","url":"https://www.hanwhadirect.com/"}&lt;/script&gt;</t>
         </is>
       </c>
       <c r="I6" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: 완성 robots.txt (/cmcom/·관리자·검색결과 Disallow)
- handoff/robots.txt 완성본 추가: Yeti·Googlebot·Daumoa 허용 + 사이트맵 2종
  Disallow /cmcom/(브릿지)·/admin//manager//mng/(관리자)·/search·검색 파라미터
- 툴 robots To-Do·Excel/PPT 태깅가이드도 동일 규칙 반영
- /cmcom/ 301 리다이렉트 케이스 caveat 주석 포함

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhxZYksEXdBzqoiFpg6L1A
</commit_message>
<xml_diff>
--- a/handoff/한화손보_장기CM_태깅가이드.xlsx
+++ b/handoff/한화손보_장기CM_태깅가이드.xlsx
@@ -1345,6 +1345,14 @@
 Allow: /
 User-agent: *
 Allow: /
+Disallow: /cmcom/
+Disallow: /admin/
+Disallow: /manager/
+Disallow: /mng/
+Disallow: /search
+Disallow: /*?keyword=
+Disallow: /*?q=
+Sitemap: https://m.hanwhadirect.com/sitemap.xml
 Sitemap: https://www.hanwhadirect.com/sitemap.xml</t>
         </is>
       </c>

</xml_diff>